<commit_message>
Điều chỉnh mô hình theo 3 nhóm hiện có của phòng
Quản lý dịch vụ (6) · Phát triển dịch vụ mới (3) · Thanh toán & quản lý hợp đồng (3);
bổ sung điểm bàn giao giữa các nhóm và đầu mối phối hợp với đơn vị ngoài phòng.
Cập nhật kế hoạch 90 ngày, file Excel, bản Word và agent vas-org-advisor.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CJdQqG1HKotrMGUKumYzgB
</commit_message>
<xml_diff>
--- a/docs/to-chuc-vas/03-bang-phan-cong-KPI-nang-luc.xlsx
+++ b/docs/to-chuc-vas/03-bang-phan-cong-KPI-nang-luc.xlsx
@@ -504,17 +504,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>QL1</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>A. Sản phẩm &amp; Tăng trưởng</t>
+          <t>1. Quản lý dịch vụ</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Trưởng nhóm A + Chủ DV Bundle</t>
+          <t>Trưởng nhóm + quản lý DV Bundle</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -534,27 +534,27 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>QL2</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>A. Sản phẩm &amp; Tăng trưởng</t>
+          <t>1. Quản lý dịch vụ</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Chủ DV SMS MO/MT sub + Thông tin giải trí</t>
+          <t>Quản lý DV SMS MO/MT subscription</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>SMS MO/MT sub; Thông tin giải trí</t>
+          <t>SMS MO/MT sub; dự phòng TTGT</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Người cũ</t>
+          <t>Người mới đi kèm DV / người cũ</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr"/>
@@ -564,27 +564,27 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>QL3</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>A. Sản phẩm &amp; Tăng trưởng</t>
+          <t>1. Quản lý dịch vụ</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Chủ DV Video + Game</t>
+          <t>Quản lý DV Thông tin giải trí</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Video; Game</t>
+          <t>Thông tin giải trí; dự phòng SMS</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Người cũ</t>
+          <t>Người mới đi kèm DV / người cũ</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
@@ -594,27 +594,27 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>QL4</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>A. Sản phẩm &amp; Tăng trưởng</t>
+          <t>1. Quản lý dịch vụ</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Tăng trưởng &amp; kênh bán (khuyến mại, upsell, tiếp thị)</t>
+          <t>Quản lý DV Video</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Dự phòng Bundle</t>
+          <t>Video; dự phòng Game</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Người mới</t>
+          <t>Người mới đi kèm DV / người cũ</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr"/>
@@ -624,27 +624,27 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>QL5</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>B. Vận hành – Chất lượng – Khiếu nại</t>
+          <t>1. Quản lý dịch vụ</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Trưởng nhóm B + Giám sát hệ thống &amp; sự cố</t>
+          <t>Quản lý DV Game</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Tất cả</t>
+          <t>Game; dự phòng Video</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Người cũ</t>
+          <t>Người mới đi kèm DV / người cũ</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr"/>
@@ -654,17 +654,17 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>QL6</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>B. Vận hành – Chất lượng – Khiếu nại</t>
+          <t>1. Quản lý dịch vụ</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Khiếu nại &amp; hoàn tiền</t>
+          <t>Số liệu &amp; kiểm soát chất lượng; đầu mối Kỹ thuật, CSKH</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -684,27 +684,27 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>PT1</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>B. Vận hành – Chất lượng – Khiếu nại</t>
+          <t>2. Phát triển dịch vụ mới</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Kiểm soát tuân thủ (kịch bản, tin nhắn, đăng ký/hủy)</t>
+          <t>Trưởng nhóm: nghiên cứu thị trường, lộ trình, thẩm định ý tưởng</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Dự phòng SMS MO/MT</t>
+          <t>DV mới</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Người mới</t>
+          <t>Người cũ</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr"/>
@@ -714,27 +714,27 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>PT2</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>B. Vận hành – Chất lượng – Khiếu nại</t>
+          <t>2. Phát triển dịch vụ mới</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Kiểm thử &amp; chất lượng (UAT, test trừ cước định kỳ)</t>
+          <t>Triển khai DV mới nhóm Bundle/Video/Game (KBDV, UAT, công văn)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Dự phòng Video</t>
+          <t>Dự phòng Bundle</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Người mới</t>
+          <t>Người cũ/mới</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr"/>
@@ -744,27 +744,27 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>PT3</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>C. Đối tác – Dữ liệu – PMO</t>
+          <t>2. Phát triển dịch vụ mới</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Trưởng nhóm C + Quản lý đối tác CP &amp; hợp đồng</t>
+          <t>Triển khai DV mới nhóm SMS/nội dung; thẩm định hồ sơ CP</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Dự phòng Game</t>
+          <t>DV mới</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Người cũ</t>
+          <t>Người cũ/mới</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr"/>
@@ -774,17 +774,17 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>TT1</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>C. Đối tác – Dữ liệu – PMO</t>
+          <t>3. Thanh toán &amp; quản lý hợp đồng</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Đối soát &amp; thanh toán doanh thu chia sẻ</t>
+          <t>Trưởng nhóm: ký mới, gia hạn, phụ lục, thanh lý hợp đồng; đầu mối Pháp chế</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -794,7 +794,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Người cũ (cẩn thận nhất)</t>
+          <t>Người cũ</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr"/>
@@ -804,27 +804,27 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>TT2</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>C. Đối tác – Dữ liệu – PMO</t>
+          <t>3. Thanh toán &amp; quản lý hợp đồng</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Phân tích dữ liệu &amp; báo cáo</t>
+          <t>Đối soát doanh thu chia sẻ</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Tất cả</t>
+          <t>Tất cả; dự phòng QL6</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Người cũ/mới</t>
+          <t>Người cũ (cẩn thận nhất)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr"/>
@@ -834,27 +834,27 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>TT3</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>C. Đối tác – Dữ liệu – PMO</t>
+          <t>3. Thanh toán &amp; quản lý hợp đồng</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>PMO: triển khai DV mới (KBDV, UAT, công văn)</t>
+          <t>Thanh toán, công nợ, chứng từ; đầu mối Kế toán</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Dự phòng Thông tin giải trí</t>
+          <t>Tất cả</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Người mới</t>
+          <t>Người cũ/mới</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr"/>
@@ -872,7 +872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -924,17 +924,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>QL1</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Trưởng nhóm A + Chủ DV Bundle</t>
+          <t>Trưởng nhóm + quản lý DV Bundle</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Doanh thu DV so kế hoạch</t>
+          <t>Doanh thu nhóm DV đang chạy so kế hoạch</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
@@ -945,13 +945,13 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>QL1</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr"/>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Thuê bao active &amp; churn</t>
+          <t>Doanh thu Bundle</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
@@ -962,13 +962,13 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>QL1</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr"/>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Tỷ lệ khiếu nại DV</t>
+          <t>Báo cáo/đề xuất danh mục đúng hạn</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
@@ -979,12 +979,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>QL2</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Chủ DV SMS MO/MT sub + Thông tin giải trí</t>
+          <t>Quản lý DV SMS MO/MT subscription</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1000,7 +1000,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>QL2</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr"/>
@@ -1017,7 +1017,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>QL2</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr"/>
@@ -1034,12 +1034,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>QL3</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Chủ DV Video + Game</t>
+          <t>Quản lý DV Thông tin giải trí</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1055,7 +1055,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>QL3</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr"/>
@@ -1072,7 +1072,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>QL3</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr"/>
@@ -1089,17 +1089,17 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>QL4</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Tăng trưởng &amp; kênh bán (khuyến mại, upsell, tiếp thị)</t>
+          <t>Quản lý DV Video</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Thuê bao mới còn giữ sau 30 ngày</t>
+          <t>Doanh thu DV so kế hoạch</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
@@ -1110,13 +1110,13 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>QL4</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr"/>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Doanh thu / chi phí khuyến mại</t>
+          <t>Thuê bao active &amp; churn</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
@@ -1127,13 +1127,13 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>QL4</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr"/>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Tỷ lệ chuyển đổi chiến dịch</t>
+          <t>Tỷ lệ khiếu nại DV</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
@@ -1144,17 +1144,17 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>QL5</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Trưởng nhóm B + Giám sát hệ thống &amp; sự cố</t>
+          <t>Quản lý DV Game</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Thời gian phát hiện → khắc phục sự cố</t>
+          <t>Doanh thu DV so kế hoạch</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
@@ -1165,13 +1165,13 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>QL5</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr"/>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Số sự cố lặp lại</t>
+          <t>Thuê bao active &amp; churn</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
@@ -1182,13 +1182,13 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>QL5</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr"/>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>% thời gian DV hoạt động</t>
+          <t>Tỷ lệ khiếu nại DV</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
@@ -1199,17 +1199,17 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>QL6</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Khiếu nại &amp; hoàn tiền</t>
+          <t>Số liệu &amp; kiểm soát chất lượng; đầu mối Kỹ thuật, CSKH</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>% khiếu nại đúng hạn</t>
+          <t>Báo cáo đúng hạn, chính xác</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
@@ -1220,13 +1220,13 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>QL6</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr"/>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Thời gian xử lý TB</t>
+          <t>Số CP/kịch bản kiểm tra/tháng</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
@@ -1237,13 +1237,13 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>QL6</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr"/>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Tỷ lệ khiếu nại lặp lại</t>
+          <t>Bất thường phát hiện trước khi bị phản ánh</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
@@ -1254,17 +1254,17 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>PT1</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Kiểm soát tuân thủ (kịch bản, tin nhắn, đăng ký/hủy)</t>
+          <t>Trưởng nhóm: nghiên cứu thị trường, lộ trình, thẩm định ý tưởng</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Số CP/kịch bản kiểm tra/tháng</t>
+          <t>Doanh thu từ DV mới (12 tháng đầu)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
@@ -1275,13 +1275,13 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>PT1</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr"/>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Vi phạm phát hiện sớm</t>
+          <t>Số DV mới ra mắt đúng kế hoạch</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
@@ -1292,13 +1292,13 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>PT1</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr"/>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>0 vi phạm tin nhắn rác</t>
+          <t>% DV mới đạt chỉ tiêu sau 6 tháng</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
@@ -1309,17 +1309,17 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>PT2</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Kiểm thử &amp; chất lượng (UAT, test trừ cước định kỳ)</t>
+          <t>Triển khai DV mới nhóm Bundle/Video/Game (KBDV, UAT, công văn)</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>% DV được test trừ cước định kỳ</t>
+          <t>% dự án đúng hạn</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr"/>
@@ -1330,13 +1330,13 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>PT2</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr"/>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Lỗi lọt sau UAT</t>
+          <t>Hồ sơ đạt ngay lần đầu</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr"/>
@@ -1347,13 +1347,13 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>PT2</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr"/>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Đúng hạn UAT</t>
+          <t>Lỗi phát sinh sau ra mắt</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr"/>
@@ -1364,17 +1364,17 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>PT3</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Trưởng nhóm C + Quản lý đối tác CP &amp; hợp đồng</t>
+          <t>Triển khai DV mới nhóm SMS/nội dung; thẩm định hồ sơ CP</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>% hợp đồng đủ hồ sơ, còn hiệu lực</t>
+          <t>% dự án đúng hạn</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr"/>
@@ -1385,13 +1385,13 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>PT3</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr"/>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Điểm đánh giá CP</t>
+          <t>Hồ sơ đạt ngay lần đầu</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr"/>
@@ -1402,13 +1402,13 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>PT3</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr"/>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Doanh thu từ CP mới</t>
+          <t>Lỗi phát sinh sau ra mắt</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr"/>
@@ -1419,17 +1419,17 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>TT1</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Đối soát &amp; thanh toán doanh thu chia sẻ</t>
+          <t>Trưởng nhóm: ký mới, gia hạn, phụ lục, thanh lý hợp đồng; đầu mối Pháp chế</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Chênh lệch đối soát &lt; 1%</t>
+          <t>% hợp đồng còn hiệu lực, đủ hồ sơ</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr"/>
@@ -1440,13 +1440,13 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>TT1</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr"/>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Đối soát đúng hạn</t>
+          <t>0 hợp đồng hết hạn mà DV vẫn chạy</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr"/>
@@ -1457,13 +1457,13 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>TT1</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr"/>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>0 sai sót thanh toán</t>
+          <t>Thời gian ký hợp đồng/phụ lục</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr"/>
@@ -1474,17 +1474,17 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>TT2</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Phân tích dữ liệu &amp; báo cáo</t>
+          <t>Đối soát doanh thu chia sẻ</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Báo cáo đúng hạn</t>
+          <t>Chênh lệch đối soát &lt; 1%</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr"/>
@@ -1495,13 +1495,13 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>TT2</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr"/>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Độ chính xác số liệu</t>
+          <t>Đối soát đúng hạn</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr"/>
@@ -1512,13 +1512,13 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>TT2</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr"/>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Số cảnh báo bất thường sớm</t>
+          <t>Số kỳ đối soát còn treo</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr"/>
@@ -1529,17 +1529,17 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>TT3</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>PMO: triển khai DV mới (KBDV, UAT, công văn)</t>
+          <t>Thanh toán, công nợ, chứng từ; đầu mối Kế toán</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>% dự án đúng hạn</t>
+          <t>Thanh toán đúng hạn</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr"/>
@@ -1550,19 +1550,36 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>TT3</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr"/>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Hồ sơ đạt ngay lần đầu</t>
+          <t>0 sai sót chi trả</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="2" t="inlineStr"/>
       <c r="G36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>TT3</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr"/>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Công nợ quá hạn giảm</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr"/>
+      <c r="E37" s="2" t="inlineStr"/>
+      <c r="F37" s="2" t="inlineStr"/>
+      <c r="G37" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1635,12 +1652,12 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Đối soát, tài chính</t>
+          <t>Triển khai DV mới (KBDV, UAT)</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Quản lý đối tác CP</t>
+          <t>Quản lý hợp đồng, đối tác CP</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
@@ -1655,7 +1672,7 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Tuân thủ/pháp lý</t>
+          <t>Đối soát, thanh toán</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
@@ -2069,7 +2086,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Hệ thống &amp; tài khoản quản trị (đã đổi mật khẩu)</t>
+          <t>Hệ thống, tài khoản quản trị; đầu mối Kỹ thuật/CSKH/Kinh doanh</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr"/>
@@ -2169,7 +2186,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Chủ DV</t>
+          <t>Người quản lý</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -2206,12 +2223,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>QL1</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>PT2</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
@@ -2230,12 +2247,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>QL2</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>QL3</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
@@ -2254,12 +2271,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>QL3</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>QL2</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
@@ -2278,12 +2295,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>QL4</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>QL5</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
@@ -2302,12 +2319,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>QL5</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>QL4</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>

</xml_diff>